<commit_message>
add Upload function: TReportSpec
</commit_message>
<xml_diff>
--- a/src/Fims.Web/Server/FimsTReportSpecsRepository/FimsTReportSpecs_Qual Sheet Sample_20221226.xlsx
+++ b/src/Fims.Web/Server/FimsTReportSpecsRepository/FimsTReportSpecs_Qual Sheet Sample_20221226.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FIMS\src\Fims.Web\Server\FimsTReportSpecsRepository\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\00FST\2023-01-19\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F31B983-ED8D-4EEA-A71E-0F270E4FE702}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5428EEA1-C75E-406F-A301-3120557D1B91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-93" yWindow="-93" windowWidth="25786" windowHeight="13866" xr2:uid="{D9BF5964-006F-4AEF-9009-C25D32BABE45}"/>
   </bookViews>
@@ -607,6 +607,10 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
+    <t>4044-Ch1</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
     <t>4044-Ch2</t>
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
@@ -655,6 +659,10 @@
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
+    <t>1008-Ch2</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
     <t>1008-Ch3</t>
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
@@ -731,6 +739,9 @@
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
+    <t>5010-Ch2</t>
+  </si>
+  <si>
     <t>5010-Ch3</t>
   </si>
   <si>
@@ -779,6 +790,10 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
+    <t>5033-Ch1</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
     <t>5033-Ch2</t>
   </si>
   <si>
@@ -820,6 +835,10 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
+    <t>5020-Ch1</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
     <t>5020-Ch2</t>
   </si>
   <si>
@@ -892,6 +911,10 @@
   </si>
   <si>
     <t>동작 (9.5)</t>
+  </si>
+  <si>
+    <t>5008-Ch1</t>
+    <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
     <t>5008-Ch2</t>
@@ -1124,6 +1147,13 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
+    <t>4013-Ch1</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>4013-Ch2</t>
+  </si>
+  <si>
     <t>4013-Ch3</t>
   </si>
   <si>
@@ -1335,6 +1365,16 @@
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
+    <t>8005-Ch1</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>8005-Ch2</t>
+  </si>
+  <si>
+    <t>8005-Ch3</t>
+  </si>
+  <si>
     <t>모니터링 통신 TEST</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
@@ -1515,50 +1555,6 @@
   </si>
   <si>
     <t>$!$-2034-Ch3</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>$!$-4044-Ch1</t>
-    <phoneticPr fontId="7" type="noConversion"/>
-  </si>
-  <si>
-    <t>$!$-5010-Ch2</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>$!$-1008-Ch2</t>
-    <phoneticPr fontId="7" type="noConversion"/>
-  </si>
-  <si>
-    <t>$!$-5008-Ch1</t>
-    <phoneticPr fontId="7" type="noConversion"/>
-  </si>
-  <si>
-    <t>$!$-5020-Ch1</t>
-    <phoneticPr fontId="7" type="noConversion"/>
-  </si>
-  <si>
-    <t>$!$-5033-Ch1</t>
-    <phoneticPr fontId="7" type="noConversion"/>
-  </si>
-  <si>
-    <t>$!$-4013-Ch1</t>
-    <phoneticPr fontId="7" type="noConversion"/>
-  </si>
-  <si>
-    <t>$!$-4013-Ch2</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>$!$-8005-Ch1</t>
-    <phoneticPr fontId="7" type="noConversion"/>
-  </si>
-  <si>
-    <t>$!$-8005-Ch2</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>$!$-8005-Ch3</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -2189,6 +2185,132 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
@@ -2222,133 +2344,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
   </cellXfs>
@@ -2837,442 +2833,442 @@
   <sheetData>
     <row r="1" spans="2:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.65"/>
     <row r="2" spans="2:15" ht="12" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B2" s="52" t="s">
+      <c r="B2" s="94" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="53"/>
-      <c r="D2" s="53"/>
-      <c r="E2" s="53"/>
-      <c r="F2" s="53"/>
-      <c r="G2" s="53"/>
-      <c r="H2" s="53"/>
-      <c r="I2" s="53"/>
-      <c r="J2" s="53"/>
-      <c r="K2" s="53"/>
-      <c r="L2" s="53"/>
-      <c r="M2" s="53"/>
-      <c r="N2" s="53"/>
-      <c r="O2" s="54"/>
+      <c r="C2" s="95"/>
+      <c r="D2" s="95"/>
+      <c r="E2" s="95"/>
+      <c r="F2" s="95"/>
+      <c r="G2" s="95"/>
+      <c r="H2" s="95"/>
+      <c r="I2" s="95"/>
+      <c r="J2" s="95"/>
+      <c r="K2" s="95"/>
+      <c r="L2" s="95"/>
+      <c r="M2" s="95"/>
+      <c r="N2" s="95"/>
+      <c r="O2" s="96"/>
     </row>
     <row r="3" spans="2:15" ht="12" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B3" s="55"/>
-      <c r="C3" s="56"/>
-      <c r="D3" s="56"/>
-      <c r="E3" s="56"/>
-      <c r="F3" s="56"/>
-      <c r="G3" s="56"/>
-      <c r="H3" s="56"/>
-      <c r="I3" s="56"/>
-      <c r="J3" s="56"/>
-      <c r="K3" s="56"/>
-      <c r="L3" s="56"/>
-      <c r="M3" s="56"/>
-      <c r="N3" s="56"/>
-      <c r="O3" s="57"/>
+      <c r="B3" s="97"/>
+      <c r="C3" s="98"/>
+      <c r="D3" s="98"/>
+      <c r="E3" s="98"/>
+      <c r="F3" s="98"/>
+      <c r="G3" s="98"/>
+      <c r="H3" s="98"/>
+      <c r="I3" s="98"/>
+      <c r="J3" s="98"/>
+      <c r="K3" s="98"/>
+      <c r="L3" s="98"/>
+      <c r="M3" s="98"/>
+      <c r="N3" s="98"/>
+      <c r="O3" s="99"/>
     </row>
     <row r="4" spans="2:15" ht="12" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B4" s="58"/>
-      <c r="C4" s="59"/>
-      <c r="D4" s="59"/>
-      <c r="E4" s="59"/>
-      <c r="F4" s="59"/>
-      <c r="G4" s="59"/>
-      <c r="H4" s="59"/>
-      <c r="I4" s="59"/>
-      <c r="J4" s="59"/>
-      <c r="K4" s="59"/>
-      <c r="L4" s="59"/>
-      <c r="M4" s="59"/>
-      <c r="N4" s="59"/>
-      <c r="O4" s="60"/>
+      <c r="B4" s="100"/>
+      <c r="C4" s="101"/>
+      <c r="D4" s="101"/>
+      <c r="E4" s="101"/>
+      <c r="F4" s="101"/>
+      <c r="G4" s="101"/>
+      <c r="H4" s="101"/>
+      <c r="I4" s="101"/>
+      <c r="J4" s="101"/>
+      <c r="K4" s="101"/>
+      <c r="L4" s="101"/>
+      <c r="M4" s="101"/>
+      <c r="N4" s="101"/>
+      <c r="O4" s="102"/>
     </row>
     <row r="5" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B5" s="61" t="s">
+      <c r="B5" s="103" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="63" t="s">
+      <c r="C5" s="64" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="63"/>
-      <c r="E5" s="63" t="s">
+      <c r="D5" s="64"/>
+      <c r="E5" s="64" t="s">
         <v>3</v>
       </c>
-      <c r="F5" s="63"/>
-      <c r="G5" s="63"/>
-      <c r="H5" s="63"/>
-      <c r="I5" s="63" t="s">
+      <c r="F5" s="64"/>
+      <c r="G5" s="64"/>
+      <c r="H5" s="64"/>
+      <c r="I5" s="64" t="s">
         <v>4</v>
       </c>
-      <c r="J5" s="63"/>
-      <c r="K5" s="64"/>
-      <c r="L5" s="64"/>
-      <c r="M5" s="65" t="s">
+      <c r="J5" s="64"/>
+      <c r="K5" s="91"/>
+      <c r="L5" s="91"/>
+      <c r="M5" s="92" t="s">
         <v>5</v>
       </c>
-      <c r="N5" s="63"/>
-      <c r="O5" s="63"/>
+      <c r="N5" s="64"/>
+      <c r="O5" s="64"/>
     </row>
     <row r="6" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B6" s="62"/>
-      <c r="C6" s="63" t="s">
+      <c r="B6" s="104"/>
+      <c r="C6" s="64" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="63"/>
-      <c r="E6" s="66" t="s">
-        <v>281</v>
-      </c>
-      <c r="F6" s="66"/>
-      <c r="G6" s="66"/>
-      <c r="H6" s="66"/>
-      <c r="I6" s="67" t="s">
+      <c r="D6" s="64"/>
+      <c r="E6" s="105" t="s">
+        <v>292</v>
+      </c>
+      <c r="F6" s="105"/>
+      <c r="G6" s="105"/>
+      <c r="H6" s="105"/>
+      <c r="I6" s="86" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="67"/>
-      <c r="K6" s="63"/>
-      <c r="L6" s="63"/>
-      <c r="M6" s="63"/>
-      <c r="N6" s="63"/>
-      <c r="O6" s="63"/>
+      <c r="J6" s="86"/>
+      <c r="K6" s="64"/>
+      <c r="L6" s="64"/>
+      <c r="M6" s="64"/>
+      <c r="N6" s="64"/>
+      <c r="O6" s="64"/>
     </row>
     <row r="7" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B7" s="62"/>
-      <c r="C7" s="63" t="s">
+      <c r="B7" s="104"/>
+      <c r="C7" s="64" t="s">
         <v>8</v>
       </c>
-      <c r="D7" s="63"/>
-      <c r="E7" s="63"/>
-      <c r="F7" s="63"/>
-      <c r="G7" s="63"/>
-      <c r="H7" s="63"/>
-      <c r="I7" s="63" t="s">
+      <c r="D7" s="64"/>
+      <c r="E7" s="64"/>
+      <c r="F7" s="64"/>
+      <c r="G7" s="64"/>
+      <c r="H7" s="64"/>
+      <c r="I7" s="64" t="s">
         <v>9</v>
       </c>
-      <c r="J7" s="63"/>
-      <c r="K7" s="64"/>
-      <c r="L7" s="64"/>
-      <c r="M7" s="63"/>
-      <c r="N7" s="63"/>
-      <c r="O7" s="63"/>
+      <c r="J7" s="64"/>
+      <c r="K7" s="91"/>
+      <c r="L7" s="91"/>
+      <c r="M7" s="64"/>
+      <c r="N7" s="64"/>
+      <c r="O7" s="64"/>
     </row>
     <row r="8" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B8" s="65" t="s">
+      <c r="B8" s="92" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="63" t="s">
+      <c r="C8" s="64" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="63"/>
-      <c r="E8" s="63"/>
-      <c r="F8" s="63"/>
-      <c r="G8" s="63"/>
-      <c r="H8" s="73" t="s">
+      <c r="D8" s="64"/>
+      <c r="E8" s="64"/>
+      <c r="F8" s="64"/>
+      <c r="G8" s="64"/>
+      <c r="H8" s="93" t="s">
         <v>12</v>
       </c>
-      <c r="I8" s="67" t="s">
+      <c r="I8" s="86" t="s">
         <v>11</v>
       </c>
-      <c r="J8" s="67"/>
-      <c r="K8" s="63"/>
-      <c r="L8" s="63"/>
-      <c r="M8" s="63"/>
-      <c r="N8" s="63"/>
-      <c r="O8" s="63"/>
+      <c r="J8" s="86"/>
+      <c r="K8" s="64"/>
+      <c r="L8" s="64"/>
+      <c r="M8" s="64"/>
+      <c r="N8" s="64"/>
+      <c r="O8" s="64"/>
     </row>
     <row r="9" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B9" s="63"/>
-      <c r="C9" s="63" t="s">
+      <c r="B9" s="64"/>
+      <c r="C9" s="64" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="63"/>
-      <c r="E9" s="63"/>
-      <c r="F9" s="63"/>
-      <c r="G9" s="63"/>
-      <c r="H9" s="67"/>
-      <c r="I9" s="67" t="s">
+      <c r="D9" s="64"/>
+      <c r="E9" s="64"/>
+      <c r="F9" s="64"/>
+      <c r="G9" s="64"/>
+      <c r="H9" s="86"/>
+      <c r="I9" s="86" t="s">
         <v>13</v>
       </c>
-      <c r="J9" s="67"/>
-      <c r="K9" s="63"/>
-      <c r="L9" s="63"/>
-      <c r="M9" s="63"/>
-      <c r="N9" s="63"/>
-      <c r="O9" s="63"/>
+      <c r="J9" s="86"/>
+      <c r="K9" s="64"/>
+      <c r="L9" s="64"/>
+      <c r="M9" s="64"/>
+      <c r="N9" s="64"/>
+      <c r="O9" s="64"/>
     </row>
     <row r="10" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B10" s="63"/>
-      <c r="C10" s="70" t="s">
+      <c r="B10" s="64"/>
+      <c r="C10" s="88" t="s">
         <v>14</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="63"/>
-      <c r="F10" s="63"/>
-      <c r="G10" s="63"/>
-      <c r="H10" s="67"/>
-      <c r="I10" s="72" t="s">
+      <c r="E10" s="64"/>
+      <c r="F10" s="64"/>
+      <c r="G10" s="64"/>
+      <c r="H10" s="86"/>
+      <c r="I10" s="90" t="s">
         <v>14</v>
       </c>
       <c r="J10" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="K10" s="63"/>
-      <c r="L10" s="63"/>
-      <c r="M10" s="63"/>
-      <c r="N10" s="63"/>
-      <c r="O10" s="63"/>
+      <c r="K10" s="64"/>
+      <c r="L10" s="64"/>
+      <c r="M10" s="64"/>
+      <c r="N10" s="64"/>
+      <c r="O10" s="64"/>
     </row>
     <row r="11" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B11" s="63"/>
-      <c r="C11" s="71"/>
+      <c r="B11" s="64"/>
+      <c r="C11" s="89"/>
       <c r="D11" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E11" s="63"/>
-      <c r="F11" s="63"/>
-      <c r="G11" s="63"/>
-      <c r="H11" s="67"/>
-      <c r="I11" s="72"/>
+      <c r="E11" s="64"/>
+      <c r="F11" s="64"/>
+      <c r="G11" s="64"/>
+      <c r="H11" s="86"/>
+      <c r="I11" s="90"/>
       <c r="J11" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="K11" s="63"/>
-      <c r="L11" s="63"/>
-      <c r="M11" s="63"/>
-      <c r="N11" s="63"/>
-      <c r="O11" s="63"/>
+      <c r="K11" s="64"/>
+      <c r="L11" s="64"/>
+      <c r="M11" s="64"/>
+      <c r="N11" s="64"/>
+      <c r="O11" s="64"/>
     </row>
     <row r="12" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B12" s="63"/>
-      <c r="C12" s="71"/>
+      <c r="B12" s="64"/>
+      <c r="C12" s="89"/>
       <c r="D12" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E12" s="63"/>
-      <c r="F12" s="63"/>
-      <c r="G12" s="63"/>
-      <c r="H12" s="67"/>
-      <c r="I12" s="72"/>
+      <c r="E12" s="64"/>
+      <c r="F12" s="64"/>
+      <c r="G12" s="64"/>
+      <c r="H12" s="86"/>
+      <c r="I12" s="90"/>
       <c r="J12" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="K12" s="63"/>
-      <c r="L12" s="63"/>
-      <c r="M12" s="63"/>
-      <c r="N12" s="63"/>
-      <c r="O12" s="63"/>
+      <c r="K12" s="64"/>
+      <c r="L12" s="64"/>
+      <c r="M12" s="64"/>
+      <c r="N12" s="64"/>
+      <c r="O12" s="64"/>
     </row>
     <row r="13" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B13" s="63"/>
-      <c r="C13" s="71"/>
+      <c r="B13" s="64"/>
+      <c r="C13" s="89"/>
       <c r="D13" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E13" s="63"/>
-      <c r="F13" s="63"/>
-      <c r="G13" s="63"/>
-      <c r="H13" s="67"/>
-      <c r="I13" s="72"/>
+      <c r="E13" s="64"/>
+      <c r="F13" s="64"/>
+      <c r="G13" s="64"/>
+      <c r="H13" s="86"/>
+      <c r="I13" s="90"/>
       <c r="J13" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="K13" s="63"/>
-      <c r="L13" s="63"/>
-      <c r="M13" s="63"/>
-      <c r="N13" s="63"/>
-      <c r="O13" s="63"/>
+      <c r="K13" s="64"/>
+      <c r="L13" s="64"/>
+      <c r="M13" s="64"/>
+      <c r="N13" s="64"/>
+      <c r="O13" s="64"/>
     </row>
     <row r="14" spans="2:15" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B14" s="67" t="s">
+      <c r="B14" s="86" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="67"/>
-      <c r="D14" s="67"/>
-      <c r="E14" s="67"/>
+      <c r="C14" s="86"/>
+      <c r="D14" s="86"/>
+      <c r="E14" s="86"/>
       <c r="F14" s="3"/>
-      <c r="G14" s="68" t="s">
+      <c r="G14" s="76" t="s">
         <v>19</v>
       </c>
-      <c r="H14" s="68"/>
-      <c r="I14" s="69" t="s">
+      <c r="H14" s="76"/>
+      <c r="I14" s="87" t="s">
         <v>20</v>
       </c>
-      <c r="J14" s="69"/>
-      <c r="K14" s="69"/>
-      <c r="L14" s="69"/>
-      <c r="M14" s="63"/>
-      <c r="N14" s="63"/>
-      <c r="O14" s="63"/>
+      <c r="J14" s="87"/>
+      <c r="K14" s="87"/>
+      <c r="L14" s="87"/>
+      <c r="M14" s="64"/>
+      <c r="N14" s="64"/>
+      <c r="O14" s="64"/>
     </row>
     <row r="15" spans="2:15" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B15" s="74" t="s">
+      <c r="B15" s="79" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="74"/>
-      <c r="D15" s="74"/>
-      <c r="E15" s="74"/>
-      <c r="F15" s="68" t="s">
+      <c r="C15" s="79"/>
+      <c r="D15" s="79"/>
+      <c r="E15" s="79"/>
+      <c r="F15" s="76" t="s">
         <v>22</v>
       </c>
-      <c r="G15" s="68"/>
-      <c r="H15" s="68"/>
-      <c r="I15" s="68"/>
-      <c r="J15" s="75" t="s">
+      <c r="G15" s="76"/>
+      <c r="H15" s="76"/>
+      <c r="I15" s="76"/>
+      <c r="J15" s="80" t="s">
         <v>23</v>
       </c>
-      <c r="K15" s="75"/>
-      <c r="L15" s="75"/>
-      <c r="M15" s="63"/>
-      <c r="N15" s="63"/>
-      <c r="O15" s="63"/>
+      <c r="K15" s="80"/>
+      <c r="L15" s="80"/>
+      <c r="M15" s="64"/>
+      <c r="N15" s="64"/>
+      <c r="O15" s="64"/>
     </row>
     <row r="16" spans="2:15" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B16" s="74"/>
-      <c r="C16" s="74"/>
-      <c r="D16" s="74"/>
-      <c r="E16" s="74"/>
-      <c r="F16" s="68" t="s">
+      <c r="B16" s="79"/>
+      <c r="C16" s="79"/>
+      <c r="D16" s="79"/>
+      <c r="E16" s="79"/>
+      <c r="F16" s="76" t="s">
         <v>24</v>
       </c>
-      <c r="G16" s="68"/>
-      <c r="H16" s="76" t="s">
-        <v>282</v>
-      </c>
-      <c r="I16" s="76"/>
+      <c r="G16" s="76"/>
+      <c r="H16" s="81" t="s">
+        <v>293</v>
+      </c>
+      <c r="I16" s="81"/>
       <c r="J16" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="K16" s="68"/>
-      <c r="L16" s="68"/>
-      <c r="M16" s="63"/>
-      <c r="N16" s="63"/>
-      <c r="O16" s="63"/>
+      <c r="K16" s="76"/>
+      <c r="L16" s="76"/>
+      <c r="M16" s="64"/>
+      <c r="N16" s="64"/>
+      <c r="O16" s="64"/>
     </row>
     <row r="17" spans="2:15" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B17" s="74"/>
-      <c r="C17" s="74"/>
-      <c r="D17" s="74"/>
-      <c r="E17" s="74"/>
-      <c r="F17" s="68" t="s">
+      <c r="B17" s="79"/>
+      <c r="C17" s="79"/>
+      <c r="D17" s="79"/>
+      <c r="E17" s="79"/>
+      <c r="F17" s="76" t="s">
         <v>25</v>
       </c>
-      <c r="G17" s="68"/>
-      <c r="H17" s="77" t="s">
-        <v>283</v>
-      </c>
-      <c r="I17" s="80" t="s">
+      <c r="G17" s="76"/>
+      <c r="H17" s="82" t="s">
+        <v>294</v>
+      </c>
+      <c r="I17" s="71" t="s">
         <v>26</v>
       </c>
-      <c r="J17" s="83" t="s">
+      <c r="J17" s="74" t="s">
         <v>27</v>
       </c>
-      <c r="K17" s="85" t="s">
+      <c r="K17" s="70" t="s">
         <v>28</v>
       </c>
-      <c r="L17" s="80"/>
-      <c r="M17" s="63"/>
-      <c r="N17" s="63"/>
-      <c r="O17" s="63"/>
+      <c r="L17" s="71"/>
+      <c r="M17" s="64"/>
+      <c r="N17" s="64"/>
+      <c r="O17" s="64"/>
     </row>
     <row r="18" spans="2:15" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B18" s="74"/>
-      <c r="C18" s="74"/>
-      <c r="D18" s="74"/>
-      <c r="E18" s="74"/>
-      <c r="F18" s="68"/>
-      <c r="G18" s="68"/>
-      <c r="H18" s="78"/>
-      <c r="I18" s="81"/>
-      <c r="J18" s="84"/>
-      <c r="K18" s="86"/>
-      <c r="L18" s="82"/>
-      <c r="M18" s="63"/>
-      <c r="N18" s="63"/>
-      <c r="O18" s="63"/>
+      <c r="B18" s="79"/>
+      <c r="C18" s="79"/>
+      <c r="D18" s="79"/>
+      <c r="E18" s="79"/>
+      <c r="F18" s="76"/>
+      <c r="G18" s="76"/>
+      <c r="H18" s="83"/>
+      <c r="I18" s="85"/>
+      <c r="J18" s="75"/>
+      <c r="K18" s="72"/>
+      <c r="L18" s="73"/>
+      <c r="M18" s="64"/>
+      <c r="N18" s="64"/>
+      <c r="O18" s="64"/>
     </row>
     <row r="19" spans="2:15" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B19" s="74"/>
-      <c r="C19" s="74"/>
-      <c r="D19" s="74"/>
-      <c r="E19" s="74"/>
-      <c r="F19" s="68"/>
-      <c r="G19" s="68"/>
-      <c r="H19" s="79"/>
-      <c r="I19" s="82"/>
-      <c r="J19" s="83" t="s">
+      <c r="B19" s="79"/>
+      <c r="C19" s="79"/>
+      <c r="D19" s="79"/>
+      <c r="E19" s="79"/>
+      <c r="F19" s="76"/>
+      <c r="G19" s="76"/>
+      <c r="H19" s="84"/>
+      <c r="I19" s="73"/>
+      <c r="J19" s="74" t="s">
         <v>29</v>
       </c>
-      <c r="K19" s="85" t="s">
+      <c r="K19" s="70" t="s">
         <v>28</v>
       </c>
-      <c r="L19" s="80"/>
-      <c r="M19" s="63"/>
-      <c r="N19" s="63"/>
-      <c r="O19" s="63"/>
+      <c r="L19" s="71"/>
+      <c r="M19" s="64"/>
+      <c r="N19" s="64"/>
+      <c r="O19" s="64"/>
     </row>
     <row r="20" spans="2:15" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B20" s="74"/>
-      <c r="C20" s="74"/>
-      <c r="D20" s="74"/>
-      <c r="E20" s="74"/>
-      <c r="F20" s="68" t="s">
+      <c r="B20" s="79"/>
+      <c r="C20" s="79"/>
+      <c r="D20" s="79"/>
+      <c r="E20" s="79"/>
+      <c r="F20" s="76" t="s">
         <v>30</v>
       </c>
-      <c r="G20" s="68"/>
-      <c r="H20" s="68" t="s">
+      <c r="G20" s="76"/>
+      <c r="H20" s="76" t="s">
         <v>31</v>
       </c>
-      <c r="I20" s="68"/>
-      <c r="J20" s="84"/>
-      <c r="K20" s="86"/>
-      <c r="L20" s="82"/>
-      <c r="M20" s="63"/>
-      <c r="N20" s="63"/>
-      <c r="O20" s="63"/>
+      <c r="I20" s="76"/>
+      <c r="J20" s="75"/>
+      <c r="K20" s="72"/>
+      <c r="L20" s="73"/>
+      <c r="M20" s="64"/>
+      <c r="N20" s="64"/>
+      <c r="O20" s="64"/>
     </row>
     <row r="21" spans="2:15" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B21" s="74"/>
-      <c r="C21" s="74"/>
-      <c r="D21" s="74"/>
-      <c r="E21" s="74"/>
-      <c r="F21" s="68"/>
-      <c r="G21" s="68"/>
-      <c r="H21" s="68"/>
-      <c r="I21" s="68"/>
-      <c r="J21" s="87" t="s">
+      <c r="B21" s="79"/>
+      <c r="C21" s="79"/>
+      <c r="D21" s="79"/>
+      <c r="E21" s="79"/>
+      <c r="F21" s="76"/>
+      <c r="G21" s="76"/>
+      <c r="H21" s="76"/>
+      <c r="I21" s="76"/>
+      <c r="J21" s="77" t="s">
         <v>32</v>
       </c>
-      <c r="K21" s="85" t="s">
+      <c r="K21" s="70" t="s">
         <v>28</v>
       </c>
-      <c r="L21" s="80"/>
-      <c r="M21" s="63"/>
-      <c r="N21" s="63"/>
-      <c r="O21" s="63"/>
+      <c r="L21" s="71"/>
+      <c r="M21" s="64"/>
+      <c r="N21" s="64"/>
+      <c r="O21" s="64"/>
     </row>
     <row r="22" spans="2:15" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B22" s="74"/>
-      <c r="C22" s="74"/>
-      <c r="D22" s="74"/>
-      <c r="E22" s="74"/>
-      <c r="F22" s="68"/>
-      <c r="G22" s="68"/>
-      <c r="H22" s="68"/>
-      <c r="I22" s="68"/>
-      <c r="J22" s="88"/>
-      <c r="K22" s="86"/>
-      <c r="L22" s="82"/>
-      <c r="M22" s="63"/>
-      <c r="N22" s="63"/>
-      <c r="O22" s="63"/>
+      <c r="B22" s="79"/>
+      <c r="C22" s="79"/>
+      <c r="D22" s="79"/>
+      <c r="E22" s="79"/>
+      <c r="F22" s="76"/>
+      <c r="G22" s="76"/>
+      <c r="H22" s="76"/>
+      <c r="I22" s="76"/>
+      <c r="J22" s="78"/>
+      <c r="K22" s="72"/>
+      <c r="L22" s="73"/>
+      <c r="M22" s="64"/>
+      <c r="N22" s="64"/>
+      <c r="O22" s="64"/>
     </row>
     <row r="23" spans="2:15" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B23" s="89" t="s">
+      <c r="B23" s="63" t="s">
         <v>33</v>
       </c>
-      <c r="C23" s="89"/>
-      <c r="D23" s="89"/>
-      <c r="E23" s="89"/>
+      <c r="C23" s="63"/>
+      <c r="D23" s="63"/>
+      <c r="E23" s="63"/>
       <c r="F23" s="3" t="s">
         <v>34</v>
       </c>
@@ -3305,10 +3301,10 @@
       </c>
     </row>
     <row r="24" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B24" s="90" t="s">
+      <c r="B24" s="57" t="s">
         <v>38</v>
       </c>
-      <c r="C24" s="63" t="s">
+      <c r="C24" s="64" t="s">
         <v>39</v>
       </c>
       <c r="D24" s="6" t="s">
@@ -3321,13 +3317,13 @@
         <v>42</v>
       </c>
       <c r="G24" s="9" t="s">
-        <v>294</v>
+        <v>43</v>
       </c>
       <c r="H24" s="10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="J24" s="11"/>
       <c r="K24" s="11"/>
@@ -3337,25 +3333,25 @@
       <c r="O24" s="12"/>
     </row>
     <row r="25" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B25" s="91"/>
-      <c r="C25" s="63"/>
+      <c r="B25" s="67"/>
+      <c r="C25" s="64"/>
       <c r="D25" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G25" s="13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H25" s="13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I25" s="13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J25" s="11"/>
       <c r="K25" s="11"/>
@@ -3365,9 +3361,9 @@
       <c r="O25" s="12"/>
     </row>
     <row r="26" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B26" s="91"/>
-      <c r="C26" s="63" t="s">
-        <v>48</v>
+      <c r="B26" s="67"/>
+      <c r="C26" s="64" t="s">
+        <v>49</v>
       </c>
       <c r="D26" s="6" t="s">
         <v>40</v>
@@ -3379,13 +3375,13 @@
         <v>42</v>
       </c>
       <c r="G26" s="14" t="s">
-        <v>284</v>
+        <v>295</v>
       </c>
       <c r="H26" s="14" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I26" s="14" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="J26" s="11"/>
       <c r="K26" s="11"/>
@@ -3395,25 +3391,25 @@
       <c r="O26" s="12"/>
     </row>
     <row r="27" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B27" s="91"/>
-      <c r="C27" s="63"/>
+      <c r="B27" s="67"/>
+      <c r="C27" s="64"/>
       <c r="D27" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G27" s="13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H27" s="13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I27" s="13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J27" s="11"/>
       <c r="K27" s="11"/>
@@ -3423,27 +3419,27 @@
       <c r="O27" s="12"/>
     </row>
     <row r="28" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B28" s="92"/>
+      <c r="B28" s="58"/>
       <c r="C28" s="15" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D28" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H28" s="10" t="s">
-        <v>296</v>
+        <v>56</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="J28" s="11"/>
       <c r="K28" s="11"/>
@@ -3453,29 +3449,29 @@
       <c r="O28" s="12"/>
     </row>
     <row r="29" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B29" s="93" t="s">
-        <v>56</v>
-      </c>
-      <c r="C29" s="94" t="s">
-        <v>57</v>
+      <c r="B29" s="62" t="s">
+        <v>58</v>
+      </c>
+      <c r="C29" s="68" t="s">
+        <v>59</v>
       </c>
       <c r="D29" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E29" s="16" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="G29" s="10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H29" s="10" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="I29" s="10" t="s">
-        <v>285</v>
+        <v>296</v>
       </c>
       <c r="J29" s="11"/>
       <c r="K29" s="11"/>
@@ -3485,25 +3481,25 @@
       <c r="O29" s="12"/>
     </row>
     <row r="30" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B30" s="89"/>
-      <c r="C30" s="95"/>
+      <c r="B30" s="63"/>
+      <c r="C30" s="69"/>
       <c r="D30" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E30" s="16" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F30" s="8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G30" s="13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H30" s="13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I30" s="13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J30" s="11"/>
       <c r="K30" s="11"/>
@@ -3513,25 +3509,25 @@
       <c r="O30" s="12"/>
     </row>
     <row r="31" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B31" s="89"/>
-      <c r="C31" s="95"/>
+      <c r="B31" s="63"/>
+      <c r="C31" s="69"/>
       <c r="D31" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E31" s="16" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="F31" s="17" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G31" s="10" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="H31" s="10" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I31" s="10" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J31" s="11"/>
       <c r="K31" s="11"/>
@@ -3541,25 +3537,25 @@
       <c r="O31" s="12"/>
     </row>
     <row r="32" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B32" s="89"/>
-      <c r="C32" s="95"/>
+      <c r="B32" s="63"/>
+      <c r="C32" s="69"/>
       <c r="D32" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E32" s="16" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F32" s="17" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H32" s="10" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="J32" s="11"/>
       <c r="K32" s="11"/>
@@ -3569,25 +3565,25 @@
       <c r="O32" s="12"/>
     </row>
     <row r="33" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B33" s="89"/>
-      <c r="C33" s="95"/>
+      <c r="B33" s="63"/>
+      <c r="C33" s="69"/>
       <c r="D33" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E33" s="16" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F33" s="17" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G33" s="10" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H33" s="10" t="s">
-        <v>295</v>
+        <v>78</v>
       </c>
       <c r="I33" s="10" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="J33" s="11"/>
       <c r="K33" s="11"/>
@@ -3597,25 +3593,25 @@
       <c r="O33" s="12"/>
     </row>
     <row r="34" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B34" s="89"/>
-      <c r="C34" s="95"/>
+      <c r="B34" s="63"/>
+      <c r="C34" s="69"/>
       <c r="D34" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E34" s="16" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="F34" s="17" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="G34" s="10" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="H34" s="10" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="I34" s="10" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="J34" s="11"/>
       <c r="K34" s="11"/>
@@ -3625,25 +3621,25 @@
       <c r="O34" s="12"/>
     </row>
     <row r="35" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B35" s="89"/>
-      <c r="C35" s="95"/>
+      <c r="B35" s="63"/>
+      <c r="C35" s="69"/>
       <c r="D35" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E35" s="16" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G35" s="13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H35" s="13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I35" s="13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J35" s="11"/>
       <c r="K35" s="11"/>
@@ -3653,25 +3649,25 @@
       <c r="O35" s="12"/>
     </row>
     <row r="36" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B36" s="89"/>
-      <c r="C36" s="95"/>
+      <c r="B36" s="63"/>
+      <c r="C36" s="69"/>
       <c r="D36" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E36" s="16" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="F36" s="8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G36" s="13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H36" s="13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I36" s="10" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="J36" s="11"/>
       <c r="K36" s="11"/>
@@ -3681,25 +3677,25 @@
       <c r="O36" s="12"/>
     </row>
     <row r="37" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B37" s="89"/>
-      <c r="C37" s="95"/>
+      <c r="B37" s="63"/>
+      <c r="C37" s="69"/>
       <c r="D37" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E37" s="16" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G37" s="13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H37" s="13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I37" s="10" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="J37" s="11"/>
       <c r="K37" s="11"/>
@@ -3709,25 +3705,25 @@
       <c r="O37" s="12"/>
     </row>
     <row r="38" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B38" s="89"/>
-      <c r="C38" s="95"/>
+      <c r="B38" s="63"/>
+      <c r="C38" s="69"/>
       <c r="D38" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E38" s="16" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="F38" s="8" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="G38" s="10" t="s">
-        <v>299</v>
+        <v>92</v>
       </c>
       <c r="H38" s="10" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="I38" s="10" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="J38" s="11"/>
       <c r="K38" s="11"/>
@@ -3737,25 +3733,25 @@
       <c r="O38" s="12"/>
     </row>
     <row r="39" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B39" s="89"/>
-      <c r="C39" s="95"/>
+      <c r="B39" s="63"/>
+      <c r="C39" s="69"/>
       <c r="D39" s="6" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="E39" s="16" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="F39" s="8" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="G39" s="10" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="H39" s="10" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="I39" s="10" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="J39" s="18"/>
       <c r="K39" s="18"/>
@@ -3765,61 +3761,61 @@
       <c r="O39" s="12"/>
     </row>
     <row r="40" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B40" s="89"/>
-      <c r="C40" s="94" t="s">
-        <v>97</v>
+      <c r="B40" s="63"/>
+      <c r="C40" s="68" t="s">
+        <v>101</v>
       </c>
       <c r="D40" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E40" s="16" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="F40" s="8" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="G40" s="19" t="s">
-        <v>298</v>
+        <v>104</v>
       </c>
       <c r="H40" s="19" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="I40" s="19" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="J40" s="20"/>
       <c r="K40" s="20"/>
       <c r="L40" s="20"/>
       <c r="M40" s="21" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="N40" s="6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="O40" s="6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="41" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B41" s="89"/>
-      <c r="C41" s="95"/>
+      <c r="B41" s="63"/>
+      <c r="C41" s="69"/>
       <c r="D41" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E41" s="22" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="F41" s="8" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="G41" s="19" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="H41" s="19" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="I41" s="19" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="J41" s="20"/>
       <c r="K41" s="20"/>
@@ -3829,25 +3825,25 @@
       <c r="O41" s="22"/>
     </row>
     <row r="42" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B42" s="89"/>
-      <c r="C42" s="95"/>
+      <c r="B42" s="63"/>
+      <c r="C42" s="69"/>
       <c r="D42" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E42" s="22" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="F42" s="8" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="G42" s="19" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="H42" s="19" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="I42" s="19" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="J42" s="20"/>
       <c r="K42" s="20"/>
@@ -3857,25 +3853,25 @@
       <c r="O42" s="22"/>
     </row>
     <row r="43" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B43" s="89"/>
-      <c r="C43" s="95"/>
+      <c r="B43" s="63"/>
+      <c r="C43" s="69"/>
       <c r="D43" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E43" s="22" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="F43" s="8" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="G43" s="19" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="H43" s="19" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="I43" s="19" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="J43" s="20"/>
       <c r="K43" s="20"/>
@@ -3885,25 +3881,25 @@
       <c r="O43" s="22"/>
     </row>
     <row r="44" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B44" s="89"/>
-      <c r="C44" s="95"/>
+      <c r="B44" s="63"/>
+      <c r="C44" s="69"/>
       <c r="D44" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E44" s="22" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="F44" s="8" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="G44" s="19" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="H44" s="19" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="I44" s="19" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="J44" s="20"/>
       <c r="K44" s="20"/>
@@ -3913,25 +3909,25 @@
       <c r="O44" s="22"/>
     </row>
     <row r="45" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B45" s="89"/>
-      <c r="C45" s="95"/>
+      <c r="B45" s="63"/>
+      <c r="C45" s="69"/>
       <c r="D45" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E45" s="22" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="F45" s="8" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="G45" s="19" t="s">
-        <v>297</v>
+        <v>127</v>
       </c>
       <c r="H45" s="19" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="I45" s="19" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="J45" s="20"/>
       <c r="K45" s="20"/>
@@ -3941,25 +3937,25 @@
       <c r="O45" s="22"/>
     </row>
     <row r="46" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B46" s="89"/>
-      <c r="C46" s="95"/>
+      <c r="B46" s="63"/>
+      <c r="C46" s="69"/>
       <c r="D46" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E46" s="22" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="F46" s="24" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="G46" s="19" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="H46" s="19" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="I46" s="19" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="J46" s="20"/>
       <c r="K46" s="20"/>
@@ -3969,25 +3965,25 @@
       <c r="O46" s="22"/>
     </row>
     <row r="47" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B47" s="89"/>
-      <c r="C47" s="95"/>
+      <c r="B47" s="63"/>
+      <c r="C47" s="69"/>
       <c r="D47" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E47" s="22" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="F47" s="8" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="G47" s="19" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="H47" s="19" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="I47" s="19" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="J47" s="20"/>
       <c r="K47" s="20"/>
@@ -3997,25 +3993,25 @@
       <c r="O47" s="22"/>
     </row>
     <row r="48" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B48" s="89"/>
-      <c r="C48" s="95"/>
+      <c r="B48" s="63"/>
+      <c r="C48" s="69"/>
       <c r="D48" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E48" s="22" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="F48" s="8" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="G48" s="19" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="H48" s="19" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="I48" s="19" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="J48" s="20"/>
       <c r="K48" s="20"/>
@@ -4025,59 +4021,59 @@
       <c r="O48" s="22"/>
     </row>
     <row r="49" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B49" s="89"/>
-      <c r="C49" s="95"/>
+      <c r="B49" s="63"/>
+      <c r="C49" s="69"/>
       <c r="D49" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E49" s="22" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="F49" s="8" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="G49" s="25" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="H49" s="25" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="I49" s="25" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="J49" s="20"/>
       <c r="K49" s="20"/>
       <c r="L49" s="20"/>
       <c r="M49" s="23" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="N49" s="6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="O49" s="6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="50" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B50" s="89"/>
-      <c r="C50" s="95"/>
+      <c r="B50" s="63"/>
+      <c r="C50" s="69"/>
       <c r="D50" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E50" s="22" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="F50" s="8" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="G50" s="25" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="H50" s="25" t="s">
-        <v>286</v>
+        <v>297</v>
       </c>
       <c r="I50" s="25" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="J50" s="20"/>
       <c r="K50" s="20"/>
@@ -4087,25 +4083,25 @@
       <c r="O50" s="26"/>
     </row>
     <row r="51" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B51" s="89"/>
-      <c r="C51" s="95"/>
+      <c r="B51" s="63"/>
+      <c r="C51" s="69"/>
       <c r="D51" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E51" s="22" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="F51" s="8" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="G51" s="25" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="H51" s="25" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="I51" s="25" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="J51" s="20"/>
       <c r="K51" s="20"/>
@@ -4115,59 +4111,59 @@
       <c r="O51" s="26"/>
     </row>
     <row r="52" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B52" s="89"/>
-      <c r="C52" s="95"/>
+      <c r="B52" s="63"/>
+      <c r="C52" s="69"/>
       <c r="D52" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E52" s="22" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="F52" s="27" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G52" s="28" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H52" s="28" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I52" s="28" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J52" s="20"/>
       <c r="K52" s="20"/>
       <c r="L52" s="20"/>
       <c r="M52" s="23" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="O52" s="6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="53" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B53" s="89"/>
-      <c r="C53" s="95"/>
+      <c r="B53" s="63"/>
+      <c r="C53" s="69"/>
       <c r="D53" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E53" s="22" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="F53" s="8" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="G53" s="25" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="H53" s="25" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="I53" s="25" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="J53" s="20"/>
       <c r="K53" s="20"/>
@@ -4177,25 +4173,25 @@
       <c r="O53" s="26"/>
     </row>
     <row r="54" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B54" s="89"/>
-      <c r="C54" s="95"/>
+      <c r="B54" s="63"/>
+      <c r="C54" s="69"/>
       <c r="D54" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E54" s="29" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="F54" s="24" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="G54" s="19" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="H54" s="19" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="I54" s="19" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="J54" s="20"/>
       <c r="K54" s="20"/>
@@ -4205,59 +4201,59 @@
       <c r="O54" s="26"/>
     </row>
     <row r="55" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B55" s="89"/>
-      <c r="C55" s="95"/>
+      <c r="B55" s="63"/>
+      <c r="C55" s="69"/>
       <c r="D55" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E55" s="29" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="F55" s="8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G55" s="13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H55" s="13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I55" s="13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J55" s="20"/>
       <c r="K55" s="20"/>
       <c r="L55" s="20"/>
       <c r="M55" s="23" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="N55" s="6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="O55" s="6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="56" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B56" s="89"/>
-      <c r="C56" s="95"/>
+      <c r="B56" s="63"/>
+      <c r="C56" s="69"/>
       <c r="D56" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E56" s="29" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="F56" s="24" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="G56" s="19" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="H56" s="19" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="I56" s="19" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="J56" s="20"/>
       <c r="K56" s="20"/>
@@ -4267,25 +4263,25 @@
       <c r="O56" s="26"/>
     </row>
     <row r="57" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B57" s="89"/>
-      <c r="C57" s="95"/>
+      <c r="B57" s="63"/>
+      <c r="C57" s="69"/>
       <c r="D57" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E57" s="29" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="F57" s="24" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="G57" s="19" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="H57" s="19" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="I57" s="19" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="J57" s="20"/>
       <c r="K57" s="20"/>
@@ -4295,25 +4291,25 @@
       <c r="O57" s="26"/>
     </row>
     <row r="58" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B58" s="89"/>
-      <c r="C58" s="95"/>
+      <c r="B58" s="63"/>
+      <c r="C58" s="69"/>
       <c r="D58" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E58" s="29" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="F58" s="24" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="G58" s="19" t="s">
-        <v>287</v>
+        <v>298</v>
       </c>
       <c r="H58" s="19" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="I58" s="19" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="J58" s="20"/>
       <c r="K58" s="20"/>
@@ -4323,59 +4319,59 @@
       <c r="O58" s="26"/>
     </row>
     <row r="59" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B59" s="89"/>
-      <c r="C59" s="95"/>
+      <c r="B59" s="63"/>
+      <c r="C59" s="69"/>
       <c r="D59" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E59" s="29" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="F59" s="8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G59" s="13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H59" s="13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I59" s="19" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="J59" s="20"/>
       <c r="K59" s="20"/>
       <c r="L59" s="20"/>
       <c r="M59" s="23" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="N59" s="6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="O59" s="26"/>
     </row>
     <row r="60" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B60" s="89"/>
-      <c r="C60" s="89" t="s">
-        <v>172</v>
+      <c r="B60" s="63"/>
+      <c r="C60" s="63" t="s">
+        <v>178</v>
       </c>
       <c r="D60" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E60" s="16" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="F60" s="30" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="G60" s="31" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="H60" s="31" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="I60" s="31" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="J60" s="32"/>
       <c r="K60" s="32"/>
@@ -4385,25 +4381,25 @@
       <c r="O60" s="12"/>
     </row>
     <row r="61" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B61" s="89"/>
-      <c r="C61" s="89"/>
+      <c r="B61" s="63"/>
+      <c r="C61" s="63"/>
       <c r="D61" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E61" s="16" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="F61" s="30" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="G61" s="31" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="H61" s="31" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="I61" s="31" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="J61" s="32"/>
       <c r="K61" s="32"/>
@@ -4413,25 +4409,25 @@
       <c r="O61" s="12"/>
     </row>
     <row r="62" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B62" s="89"/>
-      <c r="C62" s="89"/>
+      <c r="B62" s="63"/>
+      <c r="C62" s="63"/>
       <c r="D62" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E62" s="16" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="F62" s="30" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="G62" s="33" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="H62" s="33" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="I62" s="33" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="J62" s="32"/>
       <c r="K62" s="32"/>
@@ -4441,25 +4437,25 @@
       <c r="O62" s="12"/>
     </row>
     <row r="63" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B63" s="89"/>
-      <c r="C63" s="89"/>
+      <c r="B63" s="63"/>
+      <c r="C63" s="63"/>
       <c r="D63" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E63" s="16" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="F63" s="30" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="G63" s="9" t="s">
-        <v>300</v>
+        <v>194</v>
       </c>
       <c r="H63" s="9" t="s">
-        <v>301</v>
+        <v>195</v>
       </c>
       <c r="I63" s="9" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="J63" s="32"/>
       <c r="K63" s="32"/>
@@ -4469,25 +4465,25 @@
       <c r="O63" s="12"/>
     </row>
     <row r="64" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B64" s="89"/>
-      <c r="C64" s="89"/>
+      <c r="B64" s="63"/>
+      <c r="C64" s="63"/>
       <c r="D64" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E64" s="16" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="F64" s="34" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="G64" s="9" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="H64" s="9" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="I64" s="9" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="J64" s="32"/>
       <c r="K64" s="32"/>
@@ -4497,25 +4493,25 @@
       <c r="O64" s="12"/>
     </row>
     <row r="65" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B65" s="89"/>
-      <c r="C65" s="89"/>
+      <c r="B65" s="63"/>
+      <c r="C65" s="63"/>
       <c r="D65" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E65" s="16" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="F65" s="35" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="G65" s="9" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="H65" s="9" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="I65" s="9" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="J65" s="32"/>
       <c r="K65" s="32"/>
@@ -4525,25 +4521,25 @@
       <c r="O65" s="12"/>
     </row>
     <row r="66" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B66" s="89"/>
-      <c r="C66" s="89"/>
+      <c r="B66" s="63"/>
+      <c r="C66" s="63"/>
       <c r="D66" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E66" s="16" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="F66" s="35" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="G66" s="9" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="H66" s="9" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="I66" s="9" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="J66" s="32"/>
       <c r="K66" s="32"/>
@@ -4553,25 +4549,25 @@
       <c r="O66" s="12"/>
     </row>
     <row r="67" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B67" s="89"/>
-      <c r="C67" s="89"/>
+      <c r="B67" s="63"/>
+      <c r="C67" s="63"/>
       <c r="D67" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E67" s="22" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="F67" s="35" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="G67" s="9" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="H67" s="9" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="I67" s="9" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="J67" s="32"/>
       <c r="K67" s="32"/>
@@ -4581,25 +4577,25 @@
       <c r="O67" s="12"/>
     </row>
     <row r="68" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B68" s="89"/>
-      <c r="C68" s="89"/>
+      <c r="B68" s="63"/>
+      <c r="C68" s="63"/>
       <c r="D68" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E68" s="22" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="F68" s="8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G68" s="36" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H68" s="36" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I68" s="9" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="J68" s="32"/>
       <c r="K68" s="32"/>
@@ -4609,25 +4605,25 @@
       <c r="O68" s="12"/>
     </row>
     <row r="69" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B69" s="89"/>
-      <c r="C69" s="89"/>
+      <c r="B69" s="63"/>
+      <c r="C69" s="63"/>
       <c r="D69" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E69" s="22" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="F69" s="8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G69" s="36" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H69" s="36" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I69" s="9" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="J69" s="32"/>
       <c r="K69" s="32"/>
@@ -4637,25 +4633,25 @@
       <c r="O69" s="12"/>
     </row>
     <row r="70" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B70" s="89"/>
-      <c r="C70" s="89"/>
+      <c r="B70" s="63"/>
+      <c r="C70" s="63"/>
       <c r="D70" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E70" s="22" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="F70" s="35" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
       <c r="G70" s="9" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="H70" s="9" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="I70" s="9" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="J70" s="32"/>
       <c r="K70" s="32"/>
@@ -4665,25 +4661,25 @@
       <c r="O70" s="12"/>
     </row>
     <row r="71" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B71" s="89"/>
-      <c r="C71" s="89"/>
+      <c r="B71" s="63"/>
+      <c r="C71" s="63"/>
       <c r="D71" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E71" s="22" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="F71" s="35" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="G71" s="9" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="H71" s="9" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="I71" s="9" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="J71" s="32"/>
       <c r="K71" s="32"/>
@@ -4693,25 +4689,25 @@
       <c r="O71" s="12"/>
     </row>
     <row r="72" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B72" s="89"/>
-      <c r="C72" s="89"/>
+      <c r="B72" s="63"/>
+      <c r="C72" s="63"/>
       <c r="D72" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E72" s="22" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="F72" s="35" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="G72" s="9" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="H72" s="9" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="I72" s="9" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="J72" s="32"/>
       <c r="K72" s="32"/>
@@ -4721,25 +4717,25 @@
       <c r="O72" s="12"/>
     </row>
     <row r="73" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B73" s="89"/>
-      <c r="C73" s="89"/>
+      <c r="B73" s="63"/>
+      <c r="C73" s="63"/>
       <c r="D73" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E73" s="22" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="F73" s="37" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="G73" s="9" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="H73" s="9" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="I73" s="9" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="J73" s="32"/>
       <c r="K73" s="32"/>
@@ -4749,27 +4745,27 @@
       <c r="O73" s="12"/>
     </row>
     <row r="74" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B74" s="93" t="s">
-        <v>231</v>
-      </c>
-      <c r="C74" s="63" t="s">
-        <v>40</v>
-      </c>
-      <c r="D74" s="63"/>
+      <c r="B74" s="62" t="s">
+        <v>239</v>
+      </c>
+      <c r="C74" s="64" t="s">
+        <v>40</v>
+      </c>
+      <c r="D74" s="64"/>
       <c r="E74" s="22" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="F74" s="8" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="G74" s="9" t="s">
-        <v>290</v>
+        <v>301</v>
       </c>
       <c r="H74" s="9" t="s">
-        <v>288</v>
+        <v>299</v>
       </c>
       <c r="I74" s="9" t="s">
-        <v>289</v>
+        <v>300</v>
       </c>
       <c r="J74" s="32"/>
       <c r="K74" s="32"/>
@@ -4779,25 +4775,25 @@
       <c r="O74" s="12"/>
     </row>
     <row r="75" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B75" s="89"/>
-      <c r="C75" s="63" t="s">
-        <v>40</v>
-      </c>
-      <c r="D75" s="63"/>
+      <c r="B75" s="63"/>
+      <c r="C75" s="64" t="s">
+        <v>40</v>
+      </c>
+      <c r="D75" s="64"/>
       <c r="E75" s="22" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
       <c r="F75" s="38" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="G75" s="9" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="H75" s="9" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="I75" s="9" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="J75" s="32"/>
       <c r="K75" s="32"/>
@@ -4807,25 +4803,25 @@
       <c r="O75" s="12"/>
     </row>
     <row r="76" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B76" s="89"/>
-      <c r="C76" s="63" t="s">
-        <v>40</v>
-      </c>
-      <c r="D76" s="63"/>
+      <c r="B76" s="63"/>
+      <c r="C76" s="64" t="s">
+        <v>40</v>
+      </c>
+      <c r="D76" s="64"/>
       <c r="E76" s="22" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="F76" s="8" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
       <c r="G76" s="9" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="H76" s="9" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
       <c r="I76" s="9" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="J76" s="32"/>
       <c r="K76" s="32"/>
@@ -4835,25 +4831,25 @@
       <c r="O76" s="12"/>
     </row>
     <row r="77" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B77" s="89"/>
-      <c r="C77" s="97" t="s">
-        <v>40</v>
-      </c>
-      <c r="D77" s="98"/>
+      <c r="B77" s="63"/>
+      <c r="C77" s="65" t="s">
+        <v>40</v>
+      </c>
+      <c r="D77" s="66"/>
       <c r="E77" s="39" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="F77" s="17" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="G77" s="10" t="s">
-        <v>302</v>
+        <v>254</v>
       </c>
       <c r="H77" s="10" t="s">
-        <v>303</v>
+        <v>255</v>
       </c>
       <c r="I77" s="10" t="s">
-        <v>304</v>
+        <v>256</v>
       </c>
       <c r="J77" s="32"/>
       <c r="K77" s="32"/>
@@ -4863,25 +4859,25 @@
       <c r="O77" s="12"/>
     </row>
     <row r="78" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B78" s="89"/>
-      <c r="C78" s="97" t="s">
-        <v>40</v>
-      </c>
-      <c r="D78" s="98"/>
+      <c r="B78" s="63"/>
+      <c r="C78" s="65" t="s">
+        <v>40</v>
+      </c>
+      <c r="D78" s="66"/>
       <c r="E78" s="39" t="s">
-        <v>246</v>
+        <v>257</v>
       </c>
       <c r="F78" s="17" t="s">
-        <v>247</v>
+        <v>258</v>
       </c>
       <c r="G78" s="10" t="s">
-        <v>248</v>
+        <v>259</v>
       </c>
       <c r="H78" s="10" t="s">
-        <v>249</v>
+        <v>260</v>
       </c>
       <c r="I78" s="10" t="s">
-        <v>250</v>
+        <v>261</v>
       </c>
       <c r="J78" s="32"/>
       <c r="K78" s="32"/>
@@ -4891,25 +4887,25 @@
       <c r="O78" s="12"/>
     </row>
     <row r="79" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B79" s="89"/>
-      <c r="C79" s="97" t="s">
-        <v>40</v>
-      </c>
-      <c r="D79" s="98"/>
+      <c r="B79" s="63"/>
+      <c r="C79" s="65" t="s">
+        <v>40</v>
+      </c>
+      <c r="D79" s="66"/>
       <c r="E79" s="39" t="s">
-        <v>251</v>
+        <v>262</v>
       </c>
       <c r="F79" s="17" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G79" s="10" t="s">
-        <v>252</v>
+        <v>263</v>
       </c>
       <c r="H79" s="10" t="s">
-        <v>253</v>
+        <v>264</v>
       </c>
       <c r="I79" s="10" t="s">
-        <v>254</v>
+        <v>265</v>
       </c>
       <c r="J79" s="32"/>
       <c r="K79" s="32"/>
@@ -4919,25 +4915,25 @@
       <c r="O79" s="12"/>
     </row>
     <row r="80" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B80" s="89"/>
-      <c r="C80" s="63" t="s">
-        <v>255</v>
-      </c>
-      <c r="D80" s="63"/>
+      <c r="B80" s="63"/>
+      <c r="C80" s="64" t="s">
+        <v>266</v>
+      </c>
+      <c r="D80" s="64"/>
       <c r="E80" s="40" t="s">
-        <v>256</v>
+        <v>267</v>
       </c>
       <c r="F80" s="8" t="s">
-        <v>257</v>
+        <v>268</v>
       </c>
       <c r="G80" s="10" t="s">
-        <v>291</v>
+        <v>302</v>
       </c>
       <c r="H80" s="10" t="s">
-        <v>258</v>
+        <v>269</v>
       </c>
       <c r="I80" s="10" t="s">
-        <v>259</v>
+        <v>270</v>
       </c>
       <c r="J80" s="32"/>
       <c r="K80" s="32"/>
@@ -4947,25 +4943,25 @@
       <c r="O80" s="12"/>
     </row>
     <row r="81" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="B81" s="89"/>
-      <c r="C81" s="63" t="s">
-        <v>255</v>
-      </c>
-      <c r="D81" s="63"/>
+      <c r="B81" s="63"/>
+      <c r="C81" s="64" t="s">
+        <v>266</v>
+      </c>
+      <c r="D81" s="64"/>
       <c r="E81" s="40" t="s">
-        <v>260</v>
+        <v>271</v>
       </c>
       <c r="F81" s="8" t="s">
-        <v>261</v>
+        <v>272</v>
       </c>
       <c r="G81" s="10" t="s">
-        <v>292</v>
+        <v>303</v>
       </c>
       <c r="H81" s="10" t="s">
-        <v>262</v>
+        <v>273</v>
       </c>
       <c r="I81" s="10" t="s">
-        <v>293</v>
+        <v>304</v>
       </c>
       <c r="J81" s="32"/>
       <c r="K81" s="32"/>
@@ -4976,46 +4972,46 @@
     </row>
     <row r="82" spans="2:15" s="41" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.65">
       <c r="B82" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="C82" s="99"/>
-      <c r="D82" s="99"/>
-      <c r="E82" s="99"/>
-      <c r="F82" s="99"/>
-      <c r="G82" s="99"/>
-      <c r="H82" s="99"/>
-      <c r="I82" s="99"/>
-      <c r="J82" s="99"/>
-      <c r="K82" s="99"/>
-      <c r="L82" s="99"/>
+        <v>274</v>
+      </c>
+      <c r="C82" s="52"/>
+      <c r="D82" s="52"/>
+      <c r="E82" s="52"/>
+      <c r="F82" s="52"/>
+      <c r="G82" s="52"/>
+      <c r="H82" s="52"/>
+      <c r="I82" s="52"/>
+      <c r="J82" s="52"/>
+      <c r="K82" s="52"/>
+      <c r="L82" s="52"/>
       <c r="M82" s="12"/>
       <c r="N82" s="12"/>
       <c r="O82" s="12"/>
     </row>
     <row r="83" spans="2:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="C83" s="42" t="s">
-        <v>264</v>
+        <v>275</v>
       </c>
       <c r="D83" s="42"/>
       <c r="E83" s="43" t="s">
-        <v>265</v>
+        <v>276</v>
       </c>
       <c r="F83" s="44"/>
       <c r="G83" s="45" t="s">
-        <v>266</v>
+        <v>277</v>
       </c>
       <c r="H83" s="46"/>
       <c r="I83" s="45" t="s">
-        <v>267</v>
+        <v>278</v>
       </c>
       <c r="J83" s="46"/>
       <c r="K83" s="42" t="s">
-        <v>268</v>
+        <v>279</v>
       </c>
       <c r="L83" s="47"/>
-      <c r="M83" s="100"/>
-      <c r="N83" s="101"/>
-      <c r="O83" s="101"/>
+      <c r="M83" s="53"/>
+      <c r="N83" s="54"/>
+      <c r="O83" s="54"/>
     </row>
     <row r="84" spans="2:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="C84" s="42"/>
@@ -5028,108 +5024,122 @@
       <c r="J84" s="48"/>
       <c r="K84" s="42"/>
       <c r="L84" s="49"/>
-      <c r="M84" s="102"/>
-      <c r="N84" s="103"/>
-      <c r="O84" s="103"/>
+      <c r="M84" s="55"/>
+      <c r="N84" s="56"/>
+      <c r="O84" s="56"/>
     </row>
     <row r="85" spans="2:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.65">
       <c r="C85" s="50"/>
-      <c r="D85" s="90" t="s">
-        <v>269</v>
+      <c r="D85" s="57" t="s">
+        <v>280</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>270</v>
+        <v>281</v>
       </c>
       <c r="F85" s="2" t="s">
-        <v>271</v>
-      </c>
-      <c r="G85" s="104" t="s">
-        <v>272</v>
-      </c>
-      <c r="H85" s="105"/>
+        <v>282</v>
+      </c>
+      <c r="G85" s="59" t="s">
+        <v>283</v>
+      </c>
+      <c r="H85" s="60"/>
       <c r="I85" s="2" t="s">
-        <v>273</v>
+        <v>284</v>
       </c>
       <c r="J85" s="51"/>
       <c r="K85" s="2" t="s">
-        <v>274</v>
+        <v>285</v>
       </c>
       <c r="L85" s="26"/>
-      <c r="M85" s="102"/>
-      <c r="N85" s="103"/>
-      <c r="O85" s="103"/>
+      <c r="M85" s="55"/>
+      <c r="N85" s="56"/>
+      <c r="O85" s="56"/>
     </row>
     <row r="86" spans="2:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.65">
       <c r="C86" s="50"/>
-      <c r="D86" s="92"/>
+      <c r="D86" s="58"/>
       <c r="E86" s="2" t="s">
-        <v>275</v>
+        <v>286</v>
       </c>
       <c r="F86" s="2" t="s">
-        <v>276</v>
-      </c>
-      <c r="G86" s="104" t="s">
-        <v>277</v>
-      </c>
-      <c r="H86" s="105"/>
+        <v>287</v>
+      </c>
+      <c r="G86" s="59" t="s">
+        <v>288</v>
+      </c>
+      <c r="H86" s="60"/>
       <c r="I86" s="2" t="s">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="J86" s="51"/>
       <c r="K86" s="2" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="L86" s="26"/>
-      <c r="M86" s="102"/>
-      <c r="N86" s="103"/>
-      <c r="O86" s="103"/>
+      <c r="M86" s="55"/>
+      <c r="N86" s="56"/>
+      <c r="O86" s="56"/>
     </row>
     <row r="88" spans="2:15" x14ac:dyDescent="0.65">
-      <c r="B88" s="96" t="s">
-        <v>280</v>
-      </c>
-      <c r="C88" s="96"/>
-      <c r="D88" s="96"/>
-      <c r="E88" s="96"/>
+      <c r="B88" s="61" t="s">
+        <v>291</v>
+      </c>
+      <c r="C88" s="61"/>
+      <c r="D88" s="61"/>
+      <c r="E88" s="61"/>
     </row>
     <row r="89" spans="2:15" x14ac:dyDescent="0.65">
-      <c r="B89" s="96"/>
-      <c r="C89" s="96"/>
-      <c r="D89" s="96"/>
-      <c r="E89" s="96"/>
+      <c r="B89" s="61"/>
+      <c r="C89" s="61"/>
+      <c r="D89" s="61"/>
+      <c r="E89" s="61"/>
     </row>
     <row r="90" spans="2:15" x14ac:dyDescent="0.65">
-      <c r="B90" s="96"/>
-      <c r="C90" s="96"/>
-      <c r="D90" s="96"/>
-      <c r="E90" s="96"/>
+      <c r="B90" s="61"/>
+      <c r="C90" s="61"/>
+      <c r="D90" s="61"/>
+      <c r="E90" s="61"/>
     </row>
   </sheetData>
   <mergeCells count="78">
-    <mergeCell ref="M83:O86"/>
-    <mergeCell ref="D85:D86"/>
-    <mergeCell ref="G85:H85"/>
-    <mergeCell ref="G86:H86"/>
-    <mergeCell ref="B29:B73"/>
-    <mergeCell ref="C29:C39"/>
-    <mergeCell ref="C40:C59"/>
-    <mergeCell ref="C60:C73"/>
-    <mergeCell ref="B88:E90"/>
-    <mergeCell ref="B74:B81"/>
-    <mergeCell ref="C74:D74"/>
-    <mergeCell ref="C75:D75"/>
-    <mergeCell ref="C76:D76"/>
-    <mergeCell ref="C77:D77"/>
-    <mergeCell ref="C78:D78"/>
-    <mergeCell ref="C79:D79"/>
-    <mergeCell ref="C80:D80"/>
-    <mergeCell ref="C81:D81"/>
-    <mergeCell ref="C82:L82"/>
-    <mergeCell ref="K21:L22"/>
-    <mergeCell ref="B23:E23"/>
-    <mergeCell ref="B24:B28"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="B2:O4"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="E5:H5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="M5:O22"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="E6:H6"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="K6:L6"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="E7:H7"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="K7:L7"/>
+    <mergeCell ref="B14:E14"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="I14:L14"/>
+    <mergeCell ref="K8:L8"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="E9:G9"/>
+    <mergeCell ref="I9:J9"/>
+    <mergeCell ref="K9:L9"/>
+    <mergeCell ref="C10:C13"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="I10:I13"/>
+    <mergeCell ref="K10:L10"/>
+    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="B8:B13"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="E8:G8"/>
+    <mergeCell ref="K11:L11"/>
+    <mergeCell ref="E12:G12"/>
+    <mergeCell ref="K12:L12"/>
+    <mergeCell ref="E13:G13"/>
+    <mergeCell ref="K13:L13"/>
+    <mergeCell ref="H8:H13"/>
+    <mergeCell ref="I8:J8"/>
     <mergeCell ref="B15:E22"/>
     <mergeCell ref="F15:I15"/>
     <mergeCell ref="J15:L15"/>
@@ -5146,44 +5156,30 @@
     <mergeCell ref="F20:G22"/>
     <mergeCell ref="H20:I22"/>
     <mergeCell ref="J21:J22"/>
-    <mergeCell ref="B8:B13"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="E8:G8"/>
-    <mergeCell ref="K11:L11"/>
-    <mergeCell ref="E12:G12"/>
-    <mergeCell ref="K12:L12"/>
-    <mergeCell ref="E13:G13"/>
-    <mergeCell ref="K13:L13"/>
-    <mergeCell ref="H8:H13"/>
-    <mergeCell ref="I8:J8"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="I14:L14"/>
-    <mergeCell ref="K8:L8"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="E9:G9"/>
-    <mergeCell ref="I9:J9"/>
-    <mergeCell ref="K9:L9"/>
-    <mergeCell ref="C10:C13"/>
-    <mergeCell ref="E10:G10"/>
-    <mergeCell ref="I10:I13"/>
-    <mergeCell ref="K10:L10"/>
-    <mergeCell ref="E11:G11"/>
-    <mergeCell ref="B2:O4"/>
-    <mergeCell ref="B5:B7"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="E5:H5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="K5:L5"/>
-    <mergeCell ref="M5:O22"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="E6:H6"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="K6:L6"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="E7:H7"/>
-    <mergeCell ref="I7:J7"/>
-    <mergeCell ref="K7:L7"/>
-    <mergeCell ref="B14:E14"/>
+    <mergeCell ref="K21:L22"/>
+    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="B24:B28"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="B29:B73"/>
+    <mergeCell ref="C29:C39"/>
+    <mergeCell ref="C40:C59"/>
+    <mergeCell ref="C60:C73"/>
+    <mergeCell ref="B88:E90"/>
+    <mergeCell ref="B74:B81"/>
+    <mergeCell ref="C74:D74"/>
+    <mergeCell ref="C75:D75"/>
+    <mergeCell ref="C76:D76"/>
+    <mergeCell ref="C77:D77"/>
+    <mergeCell ref="C78:D78"/>
+    <mergeCell ref="C79:D79"/>
+    <mergeCell ref="C80:D80"/>
+    <mergeCell ref="C81:D81"/>
+    <mergeCell ref="C82:L82"/>
+    <mergeCell ref="M83:O86"/>
+    <mergeCell ref="D85:D86"/>
+    <mergeCell ref="G85:H85"/>
+    <mergeCell ref="G86:H86"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>